<commit_message>
feat(template): update Cum Tu JSST with 43 additional 5S/PDCA phrases (total 389)
</commit_message>
<xml_diff>
--- a/templates/Cum_Tu_JSST.xlsx
+++ b/templates/Cum_Tu_JSST.xlsx
@@ -450,7 +450,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -517,7 +517,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>346 cụm từ luyện thi JSST phản xạ giao tiếp công sở và đàm thoại hàng ngày kèm Furigana chuẩn, Audio tiếng Việt (Hoài My) và tiếng Nhật (Nanami).</t>
+          <t>389 cụm từ luyện thi JSST phản xạ giao tiếp công sở, phương pháp 5S, chu trình PDCA và đàm thoại hàng ngày kèm Furigana chuẩn, Audio tiếng Việt (Hoài My) và tiếng Nhật (Nanami).</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JSST, Cụm từ, Speaking, Japanese, Furigana, Skim</t>
+          <t>JSST, Cụm từ, Speaking, Japanese, Furigana, Skim, 5S, PDCA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -798,17 +798,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H347"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H390"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14690,6 +14690,1726 @@
       <c r="H347" t="inlineStr">
         <is>
           <t>何か困ったことがあれば、いつでも気軽に聞いてくださいね</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S (Sàng lọc - Sắp xếp - Sạch sẽ - Săn sóc - Sẵn sàng)</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>5S活動[かつどう]（整理[せいり]・整頓[せいとん]・清掃[せいそう]・清潔[せいけつ]・しつけ）</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S (Sàng lọc - Sắp xếp - Sạch sẽ - Săn sóc - Sẵn sàng)</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>5S活動（整理・整頓・清掃・清潔・しつけ）</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>5S活動[かつどう]（整理[せいり]・整頓[せいとん]・清掃[せいそう]・清潔[せいけつ]・しつけ）</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S (Sàng lọc - Sắp xếp - Sạch sẽ - Săn sóc - Sẵn sàng)</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>5S活動（整理・整頓・清掃・清潔・しつけ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Giữ cho nơi làm việc luôn ngăn nắp, sạch sẽ</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>職場[しょくば]をいつも整理整頓[せいりせいとん]し、きれいに保[たも]つ</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Giữ cho nơi làm việc luôn ngăn nắp, sạch sẽ</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>職場をいつも整理整頓し、きれいに保つ</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>職場[しょくば]をいつも整理整頓[せいりせいとん]し、きれいに保[たも]つ</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>Giữ cho nơi làm việc luôn ngăn nắp, sạch sẽ</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>職場をいつも整理整頓し、きれいに保つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Nâng cao ý thức cải thiện</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>改善[かいぜん]への意識[いしき]を高[たか]める</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Nâng cao ý thức cải thiện</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>改善への意識を高める</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>改善[かいぜん]への意識[いしき]を高[たか]める</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Nâng cao ý thức cải thiện</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>改善への意識を高める</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Ưu điểm là ngon và phong phú, nhược điểm là tốn kém</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>メリットは美味[おい]しくて種類[しゅるい]が多[おお]いこと、デメリットはコストがかかること</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Ưu điểm là ngon và phong phú, nhược điểm là tốn kém</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>メリットは美味しくて種類が多いこと、デメリットはコストがかかること</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>メリットは美味[おい]しくて種類[しゅるい]が多[おお]いこと、デメリットはコストがかかること</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Ưu điểm là ngon và phong phú, nhược điểm là tốn kém</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>メリットは美味しくて種類が多いこと、デメリットはコストがかかること</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Nấu ăn ở nhà vừa tiết kiệm vừa tốt cho sức khoẻ</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>自炊[じすい]は節約[せつやく]できるし、健康[けんこう]にもいい</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Nấu ăn ở nhà vừa tiết kiệm vừa tốt cho sức khoẻ</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>自炊は節約できるし、健康にもいい</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>自炊[じすい]は節約[せつやく]できるし、健康[けんこう]にもいい</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Nấu ăn ở nhà vừa tiết kiệm vừa tốt cho sức khoẻ</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>自炊は節約できるし、健康にもいい</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Hỏi xin công thức nấu ăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>作り方[つくりかた]を教[おし]えていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Hỏi xin công thức nấu ăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>作り方を教えていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>作り方[つくりかた]を教[おし]えていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Hỏi xin công thức nấu ăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>作り方を教えていただけますでしょうか</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Thích chơi bóng đá / cầu lông</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>サッカー／バドミントンをするのが好[す]きです</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Thích chơi bóng đá / cầu lông</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>サッカー／バドミントンをするのが好きです</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>サッカー／バドミントンをするのが好[す]きです</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Thích chơi bóng đá / cầu lông</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>サッカー、バドミントンをするのが好きです</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Duy trì thói quen tập thể dục hàng ngày</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>毎日[まいにち]運動[うんどう]する習慣[しゅうかん]を維持[いじ]する</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Duy trì thói quen tập thể dục hàng ngày</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>毎日運動する習慣を維持する</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>毎日[まいにち]運動[うんどう]する習慣[しゅうかん]を維持[いじ]する</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Duy trì thói quen tập thể dục hàng ngày</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>毎日運動する習慣を維持する</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Ca sĩ yêu thích</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>お気に入[きにい]りの歌手[かしゅ]</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Ca sĩ yêu thích</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>お気に入りの歌手</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>お気に入[きにい]りの歌手[かしゅ]</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Ca sĩ yêu thích</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>お気に入りの歌手</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Giọng hát tuyệt vời và truyền nhiều cảm xúc</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>歌声[うたごえ]が素晴[すば]らしく、元気[げんき]をもらえる</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Giọng hát tuyệt vời và truyền nhiều cảm xúc</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>歌声が素晴らしく、元気をもらえる</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>歌声[うたごえ]が素晴[すば]らしく、元気[げんき]をもらえる</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Giọng hát tuyệt vời và truyền nhiều cảm xúc</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>歌声が素晴らしく、元気をもらえる</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Ngọn núi đẹp nổi tiếng (như núi Phùng, Fansipan)</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>美[うつく]しい有名[ゆうめい]な山[やま]</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Ngọn núi đẹp nổi tiếng (như núi Phùng, Fansipan)</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>美しい有名な山</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>美[うつく]しい有名[ゆうめい]な山[やま]</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Ngọn núi đẹp nổi tiếng (như núi Phùng, Fansipan)</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>美しい有名な山</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Tận hưởng thiên nhiên hùng vĩ</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>豊[ゆた]かな大自然[だいしぜん]を満喫[まんきつ]する</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Tận hưởng thiên nhiên hùng vĩ</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>豊かな大自然を満喫する</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>豊[ゆた]かな大自然[だいしぜん]を満喫[まんきつ]する</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Tận hưởng thiên nhiên hùng vĩ</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>豊かな大自然を満喫する</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Giới thiệu địa điểm du lịch hấp dẫn</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>魅力的[みりょくてき]な観光地[かんこうち]を紹介[しょうかい]する</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Giới thiệu địa điểm du lịch hấp dẫn</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>魅力的な観光地を紹介する</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>魅力的[みりょくてき]な観光地[かんこうち]を紹介[しょうかい]する</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Giới thiệu địa điểm du lịch hấp dẫn</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>魅力的な観光地を紹介する</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Xin phép vắng mặt do con ốm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>子[こ]どもが病気[びょうき]のため、欠席[けっせき]させていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Xin phép vắng mặt do con ốm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>子どもが病気のため、欠席させていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>子[こ]どもが病気[びょうき]のため、欠席[けっせき]させていただけますでしょうか</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Xin phép vắng mặt do con ốm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>子どもが病気のため、欠席させていただけますでしょうか</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Báo cáo lịch trình công tác thay đổi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>出張[しゅっちょう]日程[にってい]が変更[へんこう]になりましたので、ご報告[ほうこく]いたします</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Báo cáo lịch trình công tác thay đổi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>出張日程が変更になりましたので、ご報告いたします</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>出張[しゅっちょう]日程[にってい]が変更[へんこう]になりましたので、ご報告[ほうこく]いたします</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Báo cáo lịch trình công tác thay đổi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>出張日程が変更になりましたので、ご報告いたします</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Quên mang máy tính và xin lỗi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>パソコンを忘[わす]れしまいました。大変申[たいへんもう]し訳[わけ]ございません</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Quên mang máy tính và xin lỗi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>パソコンを忘れしまいました。大変申し訳ございません</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>パソコンを忘[わす]れしまいました。大変申[たいへんもう]し訳[わけ]ございません</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Quên mang máy tính và xin lỗi (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>パソコンを忘れしまいました。大変申し訳ございません</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Xin ý kiến hướng dẫn khi không hiểu hệ thống (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>システムが分[わ]からないため、ご指導[しどう]をお願[ねが]いできますでしょうか</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Xin ý kiến hướng dẫn khi không hiểu hệ thống (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>システムが分からないため、ご指導をお願いできますでしょうか</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>システムが分[わ]からないため、ご指導[しどう]をお願[ねが]いできますでしょうか</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Xin ý kiến hướng dẫn khi không hiểu hệ thống (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>システムが分からないため、ご指導をお願いできますでしょうか</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Trình bày nguyện vọng tham gia dự án mới (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>新[あたら]しいプロジェクトに参加[さんか]させていただきたいのですが</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Trình bày nguyện vọng tham gia dự án mới (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>新しいプロジェクトに参加させていただきたいのですが</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>新[あたら]しいプロジェクトに参加[さんか]させていただきたいのですが</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Trình bày nguyện vọng tham gia dự án mới (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>新しいプロジェクトに参加させていただきたいのですが</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Từ chối khéo khi bận việc đột xuất (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>あいにく手[て]が離[はな]せないのですが</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Từ chối khéo khi bận việc đột xuất (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>あいにく手が離せないのですが</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>あいにく手[て]が離[はな]せないのですが</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>Từ chối khéo khi bận việc đột xuất (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>あいにく手が離せないのですが</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Xin phép rời phòng họp sớm / về sớm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>お先[さき]に失礼[しつれい]させていただきます</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Xin phép rời phòng họp sớm / về sớm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>お先に失礼させていただきます</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>お先[さき]に失礼[しつれい]させていただきます</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>Xin phép rời phòng họp sớm / về sớm (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>お先に失礼させていただきます</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Xử lý khi phát hiện lỗi nghiêm trọng (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>重大[じゅうだい]な不具合[ふぐあい]を発見[はっけん]いたしましたので、至急[しきゅう]ご報告[ほうこく]します</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Xử lý khi phát hiện lỗi nghiêm trọng (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>重大な不具合を発見いたしましたので、至急ご報告します</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>重大[じゅうだい]な不具合[ふぐあい]を発見[はっけん]いたしましたので、至急[しきゅう]ご報告[ほうこく]します</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Xử lý khi phát hiện lỗi nghiêm trọng (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>重大な不具合を発見いたしましたので、至急ご報告します</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Xin ý kiến giải quyết khi gặp khó khăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>今後[こんご]の対応[たいおう]について、ご指示[しじ]を仰[あお]ぎたいのですが</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Xin ý kiến giải quyết khi gặp khó khăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>今後の対応について、ご指示を仰ぎたいのですが</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>今後[こんご]の対応[たいおう]について、ご指示[しじ]を仰[あお]ぎたいのですが</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Xin ý kiến giải quyết khi gặp khó khăn (Kính ngữ)</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>今後の対応について、ご指示を仰ぎたいのですが</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Hỏi thăm người đồng nghiệp gặp khó khăn</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>何[なに]か困[こま]ったことはありませんか。お手伝[てつだ]いしましょうか</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Hỏi thăm người đồng nghiệp gặp khó khăn</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>何か困ったことはありませんか。お手伝いしましょうか</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>何[なに]か困[こま]ったことはありませんか。お手伝[てつだ]いしましょうか</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Hỏi thăm người đồng nghiệp gặp khó khăn</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>何か困ったことはありませんか。お手伝いしましょうか</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Cảm ơn vì đã giúp đỡ tận tình</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>丁寧[ていねい]にご対応[たいおう]いただき、本当[ほんとう]にありがとうございます</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Cảm ơn vì đã giúp đỡ tận tình</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>丁寧にご対応いただき、本当にありがとうございます</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>丁寧[ていねい]にご対応[たいおう]いただき、本当[ほんとう]にありがとうございます</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>Cảm ơn vì đã giúp đỡ tận tình</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>丁寧にご対応いただき、本当にありがとうございます</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S triệt để</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>5Sを徹底[てってい]する</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S triệt để</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>5Sを徹底する</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>5Sを徹底[てってい]する</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Thực hiện 5S triệt để</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>5Sを徹底する</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Sàng lọc (Loại bỏ đồ không cần thiết)</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>整理[せいり]（不要[ふよう]なものを捨[す]てる）</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Sàng lọc (Loại bỏ đồ không cần thiết)</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>整理（不要なものを捨てる）</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>整理[せいり]（不要[ふよう]なものを捨[す]てる）</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Sàng lọc (Loại bỏ đồ không cần thiết)</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>整理（不要なものを捨てる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Sắp xếp (Để đúng nơi, dễ lấy)</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>整頓[せいとん]（置き場[おきば]を決[き]め、取り出[とりだ]しやすくする）</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Sắp xếp (Để đúng nơi, dễ lấy)</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>整頓（置き場を決め、取り出しやすくする）</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>整頓[せいとん]（置き場[おきば]を決[き]め、取り出[とりだ]しやすくする）</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Sắp xếp (Để đúng nơi, dễ lấy)</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>整頓（置き場を決め、取り出しやすくする）</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Sạch sẽ (Lau chùi, dọn dẹp vệ sinh)</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>清掃[せいそう]（きれいに掃除[そうじ]する）</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Sạch sẽ (Lau chùi, dọn dẹp vệ sinh)</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>清掃（きれいに掃除する）</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>清掃[せいそう]（きれいに掃除[そうじ]する）</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Sạch sẽ (Lau chùi, dọn dẹp vệ sinh)</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>清掃（きれいに掃除する）</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Săn sóc (Duy trì trạng thái sạch sẽ)</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>清潔[せいけつ]（きれいな状態[じょうたい]を維持[いじ]する）</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Săn sóc (Duy trì trạng thái sạch sẽ)</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>清潔（きれいな状態を維持する）</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>清潔[せいけつ]（きれいな状態[じょうたい]を維持[いじ]する）</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Săn sóc (Duy trì trạng thái sạch sẽ)</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>清潔（きれいな状態を維持する）</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Sẵn sàng (Tuân thủ nghiêm ngặt quy định)</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>しつけ（ルールをしっかり守[まも]る）</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Sẵn sàng (Tuân thủ nghiêm ngặt quy định)</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>しつけ（ルールをしっかり守る）</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>しつけ（ルールをしっかり守[まも]る）</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Sẵn sàng (Tuân thủ nghiêm ngặt quy định)</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>しつけ（ルールをしっかり守る）</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Dọn dẹp bàn làm việc mỗi ngày</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>毎日[まいにち]の終[お]わりに机[つくえ]を片付[かたづ]ける</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Dọn dẹp bàn làm việc mỗi ngày</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>毎日の終わりに机を片付ける</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>毎日[まいにち]の終[お]わりに机[つくえ]を片付[かたづ]ける</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Dọn dẹp bàn làm việc mỗi ngày</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>毎日の終わりに机を片付ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Tìm đồ nhanh chóng nhờ 5S</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>5Sのおかげで物[もの]をすぐ見[み]つけられる</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Tìm đồ nhanh chóng nhờ 5S</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>5Sのおかげで物をすぐ見つけられる</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>5Sのおかげで物[もの]をすぐ見[み]つけられる</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Tìm đồ nhanh chóng nhờ 5S</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>5Sのおかげで物をすぐ見つけられる</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Giảm thiểu sai sót nhờ ngăn nắp</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>整理整頓[せいりせいとん]でミスを減[へ]らす</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Giảm thiểu sai sót nhờ ngăn nắp</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>整理整頓でミスを減らす</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>整理整頓[せいりせいとん]でミスを減[へ]らす</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Giảm thiểu sai sót nhờ ngăn nắp</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>整理整頓でミスを減らす</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Nâng cao hiệu suất nhờ môi trường sạch</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>きれいな職場[しょくば]で効率[こうりつ]が上[あ]がる</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Nâng cao hiệu suất nhờ môi trường sạch</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>きれいな職場で効率が上がる</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>きれいな職場[しょくば]で効率[こうりつ]が上[あ]がる</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Nâng cao hiệu suất nhờ môi trường sạch</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>きれいな職場で効率が上がる</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch chi tiết (Plan)</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>計画[けいかく]を立[た]てる（Plan）</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch chi tiết (Plan)</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>計画を立てる（Plan）</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>計画[けいかく]を立[た]てる（Plan）</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch chi tiết (Plan)</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>計画を立てる（Plan）</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Thực hiện theo đúng kế hoạch (Do)</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>計画[けいかく]通[とう]りに実行[じっこう]する（Do）</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Thực hiện theo đúng kế hoạch (Do)</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>計画通りに実行する（Do）</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>計画[けいかく]通[とう]りに実行[じっこう]する（Do）</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Thực hiện theo đúng kế hoạch (Do)</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>計画通りに実行する（Do）</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Kiểm tra kết quả và tiến độ (Check)</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>進捗[しんちょく]や結果[けっか]を確認[かくにん]する（Check）</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Kiểm tra kết quả và tiến độ (Check)</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>進捗や結果を確認する（Check）</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>進捗[しんちょく]や結果[けっか]を確認[かくにん]する（Check）</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>Kiểm tra kết quả và tiến độ (Check)</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>進捗や結果を確認する（Check）</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Hành động cải thiện vấn đề phát sinh (Act)</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>問題点[もんだいてん]を改善[かいぜん]する（Act）</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Hành động cải thiện vấn đề phát sinh (Act)</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>問題点を改善する（Act）</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>問題点[もんだいてん]を改善[かいぜん]する（Act）</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Hành động cải thiện vấn đề phát sinh (Act)</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>問題点を改善する（Act）</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Lặp lại chu trình PDCA để nâng cao chất lượng</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>PDCAを回[まわ]して品質[ひんしつ]を向上[こうじょう]させる</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Lặp lại chu trình PDCA để nâng cao chất lượng</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>PDCAを回して品質を向上させる</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>PDCAを回[まわ]して品質[ひんしつ]を向上[こうじょう]させる</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>Lặp lại chu trình PDCA để nâng cao chất lượng</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>PDCAを回して品質を向上させる</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Xác định rõ nguyên nhân gốc rễ</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>根本的[こんぽんてき]な原因[げんいん]を突[つ]き止[や]める</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Xác định rõ nguyên nhân gốc rễ</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>根本的な原因を突き止める</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>根本的[こんぽんてき]な原因[げんいん]を突[つ]き止[や]める</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>Xác định rõ nguyên nhân gốc rễ</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>根本的な原因を突き止める</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Đề ra biện pháp đối phó hiệu quả</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>効果的[こうかてき]な対策[たいさく]を立[た]てる</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Đề ra biện pháp đối phó hiệu quả</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>効果的な対策を立てる</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>効果的[こうかてき]な対策[たいさく]を立[た]てる</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>Đề ra biện pháp đối phó hiệu quả</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>効果的な対策を立てる</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Triển khai hành động khắc phục ngay lập tức</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>至急[しきゅう]、改善策[かいぜんさく]を実施[じっし]する</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Triển khai hành động khắc phục ngay lập tức</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>至急、改善策を実施する</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>至急[しきゅう]、改善策[かいぜんさく]を実施[じっし]する</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>Triển khai hành động khắc phục ngay lập tức</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>至急、改善策を実施する</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Chia sẻ kết quả cải tiến với toàn đội</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>改善[かいぜん]結果[けっか]をチームで共有[きょうゆう]する</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Chia sẻ kết quả cải tiến với toàn đội</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>改善結果をチームで共有する</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>改善[かいぜん]結果[けっか]をチームで共有[きょうゆう]する</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>Chia sẻ kết quả cải tiến với toàn đội</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>改善結果をチームで共有する</t>
         </is>
       </c>
     </row>
@@ -14706,7 +16426,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
feat(templates): update Cum_Tu_JSST.xlsx with 494 curated JSST collocations and furigana
</commit_message>
<xml_diff>
--- a/templates/Cum_Tu_JSST.xlsx
+++ b/templates/Cum_Tu_JSST.xlsx
@@ -450,7 +450,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -517,7 +517,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>389 cụm từ luyện thi JSST phản xạ giao tiếp công sở, phương pháp 5S, chu trình PDCA và đàm thoại hàng ngày kèm Furigana chuẩn, Audio tiếng Việt (Hoài My) và tiếng Nhật (Nanami).</t>
+          <t>494 cụm từ luyện thi JSST phản xạ giao tiếp cốt lõi theo 12 chủ đề toàn diện: công sở, kính ngữ, kỹ năng, teamwork, AI &amp; công nghệ số, môi trường, giao thông, đời sống gia đình, sức khỏe, du lịch, tiêu dùng và đa văn hóa kèm Furigana chuẩn, Audio Hoài My (VI) và Nanami (JA).</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JSST, Cụm từ, Speaking, Japanese, Furigana, Skim, 5S, PDCA</t>
+          <t>JSST, Cụm từ, Speaking, Japanese, Furigana, Skim, Collocations</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -798,8 +798,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H390"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:H495"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -16413,6 +16413,4206 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Từ chối khéo vì đã có hẹn trước</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>あいにく先約[せんやく]がございまして</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Từ chối khéo vì đã có hẹn trước</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>あいにく先約がございまして</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>あいにく先約[せんやく]がございまして</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Từ chối khéo vì đã có hẹn trước</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>あいにく先約がございまして</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Đến muộn do sự cố tàu xe</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>電車[でんしゃ]の遅延[ちえん]で遅[おく]れる</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Đến muộn do sự cố tàu xe</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>電車の遅延で遅れる</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>電車[でんしゃ]の遅延[ちえん]で遅[おく]れる</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Đến muộn do sự cố tàu xe</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>電車の遅延で遅れる</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Bàn giao công việc cẩn thận</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>業務[ぎょうむ]を引き継[ひきつ]ぐ</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Bàn giao công việc cẩn thận</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>業務を引き継ぐ</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>業務[ぎょうむ]を引き継[ひきつ]ぐ</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Bàn giao công việc cẩn thận</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>業務を引き継ぐ</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Mong anh/chị lượng thứ bỏ qua</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>何卒[なにとぞ]ご容赦[ようしゃ]ください</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Mong anh/chị lượng thứ bỏ qua</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>何卒ご容赦ください</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>何卒[なにとぞ]ご容赦[ようしゃ]ください</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Mong anh/chị lượng thứ bỏ qua</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>何卒ご容赦ください</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Sẽ gọi điện thoại lại ngay</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>折り返[おりかえ]しお電話[でんわ]いたします</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Sẽ gọi điện thoại lại ngay</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>折り返しお電話いたします</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>折り返[おりかえ]しお電話[でんわ]いたします</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Sẽ gọi điện thoại lại ngay</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>折り返しお電話いたします</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>395</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Tiến hành xử lý khẩn cấp</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>至急[しきゅう]対応[たいおう]いたします</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Tiến hành xử lý khẩn cấp</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>至急対応いたします</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>至急[しきゅう]対応[たいおう]いたします</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Tiến hành xử lý khẩn cấp</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>至急対応いたします</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>396</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Hướng tới thăng tiến sự nghiệp</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>キャリアアップを目指[めざ]す</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Hướng tới thăng tiến sự nghiệp</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>キャリアアップを目指す</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>キャリアアップを目指[めざ]す</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Hướng tới thăng tiến sự nghiệp</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>キャリアアップを目指す</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>397</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Kiên trì hoàn thành mục tiêu</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>目標[もくひょう]を達成[たっせい]する</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Kiên trì hoàn thành mục tiêu</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>目標を達成する</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>目標[もくひょう]を達成[たっせい]する</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Kiên trì hoàn thành mục tiêu</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>目標を達成する</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>398</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Rèn luyện tính tự giác quản lý</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>自己管理[じこかんり]を徹底[てってい]する</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Rèn luyện tính tự giác quản lý</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>自己管理を徹底する</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>自己管理[じこかんり]を徹底[てってい]する</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Rèn luyện tính tự giác quản lý</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>自己管理を徹底する</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>399</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Đào sâu kiến thức chuyên môn</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>専門知識[せんもんちしき]を深[ふか]める</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Đào sâu kiến thức chuyên môn</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>専門知識を深める</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>専門知識[せんもんちしき]を深[ふか]める</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Đào sâu kiến thức chuyên môn</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>専門知識を深める</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>400</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Phân bổ thời gian hợp lý</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>時間配分[じかんはいぶん]を考[かんが]える</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Phân bổ thời gian hợp lý</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>時間配分を考える</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>時間配分[じかんはいぶん]を考[かんが]える</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Phân bổ thời gian hợp lý</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>時間配分を考える</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>401</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Tạo ra thành quả cụ thể rõ nét</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>具体的[ぐたいてき]な成果[せいか]を出[だ]す</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Tạo ra thành quả cụ thể rõ nét</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>具体的な成果を出す</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>具体的[ぐたいてき]な成果[せいか]を出[だ]す</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Tạo ra thành quả cụ thể rõ nét</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>具体的な成果を出す</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>402</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Vượt qua áp lực công việc</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>プレッシャーを乗り越[のりこ]える</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Vượt qua áp lực công việc</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>プレッシャーを乗り越える</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>プレッシャーを乗り越[のりこ]える</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Vượt qua áp lực công việc</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>プレッシャーを乗り越える</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>403</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Tự tin phát huy điểm mạnh bản thân</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>自分[じぶん]の強[つよ]みを活[い]かす</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Tự tin phát huy điểm mạnh bản thân</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>自分の強みを活かす</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>自分[じぶん]の強[つよ]みを活[い]かす</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Tự tin phát huy điểm mạnh bản thân</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>自分の強みを活かす</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>404</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Bình tĩnh giải quyết mâu thuẫn</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>冷静[れいせい]に話し合[はなしあ]う</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Bình tĩnh giải quyết mâu thuẫn</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>冷静に話し合う</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>冷静[れいせい]に話し合[はなしあ]う</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Bình tĩnh giải quyết mâu thuẫn</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>冷静に話し合う</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>405</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Đưa ra ý kiến mang tính xây dựng</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>建設的[けんせつてき]な意見[いけん]を出[だ]す</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Đưa ra ý kiến mang tính xây dựng</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>建設的な意見を出す</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>建設的[けんせつてき]な意見[いけん]を出[だ]す</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Đưa ra ý kiến mang tính xây dựng</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>建設的な意見を出す</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>406</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Duy trì họp trao đổi định kỳ</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>定期的[ていきてき]にミーティングを開[ひら]く</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Duy trì họp trao đổi định kỳ</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>定期的にミーティングを開く</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>定期的[ていきてき]にミーティングを開[ひら]く</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Duy trì họp trao đổi định kỳ</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>定期的にミーティングを開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>407</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Xóa bỏ sự lệch pha trong hiểu biết</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>認識[にんしき]のズレをなくす</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Xóa bỏ sự lệch pha trong hiểu biết</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>認識のズレをなくす</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>認識[にんしき]のズレをなくす</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Xóa bỏ sự lệch pha trong hiểu biết</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>認識のズレをなくす</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>408</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Tiếp thu ý kiến phản hồi tích cực</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>フィードバックを受け入[うけい]れる</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Tiếp thu ý kiến phản hồi tích cực</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>フィードバックを受け入れる</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>フィードバックを受け入[うけい]れる</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Tiếp thu ý kiến phản hồi tích cực</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>フィードバックを受け入れる</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>409</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Đoàn kết tạo nên sức mạnh lớn</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>結束力[けっそくりょく]を強[つよ]める</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Đoàn kết tạo nên sức mạnh lớn</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>結束力を強める</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>結束力[けっそくりょく]を強[つよ]める</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>Đoàn kết tạo nên sức mạnh lớn</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>結束力を強める</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>410</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Tôn trọng sự đa dạng tính cách</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>個性[こせい]の違[ちが]いを認[みと]める</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Tôn trọng sự đa dạng tính cách</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>個性の違いを認める</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>個性[こせい]の違[ちが]いを認[みと]める</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Tôn trọng sự đa dạng tính cách</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>個性の違いを認める</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>411</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Làm chủ và sử dụng AI thông minh</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>AIを賢[かしこ]く使[つか]いこなす</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Làm chủ và sử dụng AI thông minh</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>AIを賢く使いこなす</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>AIを賢[かしこ]く使[つか]いこなす</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Làm chủ và sử dụng AI thông minh</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>AIを賢く使いこなす</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>412</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Dịch thuật đa ngôn ngữ tức thì</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>多言語[たげんご]を自動翻訳[じどうほんやく]する</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Dịch thuật đa ngôn ngữ tức thì</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>多言語を自動翻訳する</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>多言語[たげんご]を自動翻訳[じどうほんやく]する</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Dịch thuật đa ngôn ngữ tức thì</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>多言語を自動翻訳する</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>413</v>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Mở rộng ý tưởng sáng tạo mới</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>新[あたら]しいアイデアを広[ひろ]げる</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Mở rộng ý tưởng sáng tạo mới</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>新しいアイデアを広げる</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>新[あたら]しいアイデアを広[ひろ]げる</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Mở rộng ý tưởng sáng tạo mới</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>新しいアイデアを広げる</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>414</v>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Phân tích dữ liệu để ra quyết định</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>データを分析[ぶんせき]する</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Phân tích dữ liệu để ra quyết định</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>データを分析する</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>データを分析[ぶんせき]する</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>Phân tích dữ liệu để ra quyết định</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>データを分析する</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>415</v>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Rèn luyện tư duy phản biện độc lập</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>批判的[ひはんてき]思考力[しこうりょく]を磨[みが]く</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Rèn luyện tư duy phản biện độc lập</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>批判的思考力を磨く</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>批判的[ひはんてき]思考力[しこうりょく]を磨[みが]く</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Rèn luyện tư duy phản biện độc lập</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>批判的思考力を磨く</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>416</v>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Ứng dụng thuật toán tối ưu hóa</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>アルゴリズムを活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Ứng dụng thuật toán tối ưu hóa</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>アルゴリズムを活用する</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>アルゴリズムを活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Ứng dụng thuật toán tối ưu hóa</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>アルゴリズムを活用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>417</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Thích nghi nhanh với thời đại số</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>デジタル時代[じだい]に適応[てきおう]する</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Thích nghi nhanh với thời đại số</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>デジタル時代に適応する</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>デジタル時代[じだい]に適応[てきおう]する</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Thích nghi nhanh với thời đại số</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>デジタル時代に適応する</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>418</v>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Hạn chế lạm dụng smartphone</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>スマホの使[つか]いすぎを防[ふせ]ぐ</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Hạn chế lạm dụng smartphone</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>スマホの使いすぎを防ぐ</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>スマホの使[つか]いすぎを防[ふせ]ぐ</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Hạn chế lạm dụng smartphone</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>スマホの使いすぎを防ぐ</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>419</v>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Dễ dàng kết nối bạn bè phương xa</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>遠[とお]くの友人[ゆうじん]とつながる</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Dễ dàng kết nối bạn bè phương xa</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>遠くの友人とつながる</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>遠[とお]くの友人[ゆうじん]とつながる</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Dễ dàng kết nối bạn bè phương xa</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>遠くの友人とつながる</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>420</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Bảo vệ quyền riêng tư cá nhân</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>プライバシーを保護[ほご]する</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Bảo vệ quyền riêng tư cá nhân</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>プライバシーを保護する</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>プライバシーを保護[ほご]する</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>Bảo vệ quyền riêng tư cá nhân</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>プライバシーを保護する</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>421</v>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Tuân thủ văn hóa ứng xử trên mạng</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>ネットマナーを守[まも]る</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Tuân thủ văn hóa ứng xử trên mạng</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>ネットマナーを守る</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>ネットマナーを守[まも]る</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>Tuân thủ văn hóa ứng xử trên mạng</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>ネットマナーを守る</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>422</v>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Tắt bớt thông báo để tập trung</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>通知[つうち]をオフにする</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Tắt bớt thông báo để tập trung</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>通知をオフにする</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>通知[つうち]をオフにする</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>Tắt bớt thông báo để tập trung</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>通知をオフにする</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>423</v>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Cảnh giác cao trước email lừa đảo</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>詐欺[さぎ]メールに警戒[けいかい]する</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Cảnh giác cao trước email lừa đảo</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>詐欺メールに警戒する</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>詐欺[さぎ]メールに警戒[けいかい]する</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Cảnh giác cao trước email lừa đảo</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>詐欺メールに警戒する</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>424</v>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Tạm thời cai nghiện thiết bị số</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>デジタルデトックスを行[おこな]う</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Tạm thời cai nghiện thiết bị số</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>デジタルデトックスを行う</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>デジタルデトックスを行[おこな]う</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Tạm thời cai nghiện thiết bị số</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>デジタルデトックスを行う</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>425</v>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Tự chịu trách nhiệm với lời phát ngôn</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>発言[はつげん]に責任[せきにん]を持[も]つ</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Tự chịu trách nhiệm với lời phát ngôn</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>発言に責任を持つ</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>発言[はつげん]に責任[せきにん]を持[も]つ</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Tự chịu trách nhiệm với lời phát ngôn</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>発言に責任を持つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>426</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Cập nhật phần mềm hệ điều hành</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>システムを最新[さいしん]に保[たも]つ</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Cập nhật phần mềm hệ điều hành</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>システムを最新に保つ</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>システムを最新[さいしん]に保[たも]つ</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Cập nhật phần mềm hệ điều hành</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>システムを最新に保つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>427</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Tìm kiếm bạn bè cùng sở thích</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>同[おな]じ趣味[しゅみ]の仲間[なかま]を見[み]つける</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Tìm kiếm bạn bè cùng sở thích</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>同じ趣味の仲間を見つける</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>同[おな]じ趣味[しゅみ]の仲間[なかま]を見[み]つける</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Tìm kiếm bạn bè cùng sở thích</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>同じ趣味の仲間を見つける</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>428</v>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Tăng cường trồng thêm cây xanh</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>緑[みどり]や木[き]を増[ふ]やす</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Tăng cường trồng thêm cây xanh</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>緑や木を増やす</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>緑[みどり]や木[き]を増[ふ]やす</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Tăng cường trồng thêm cây xanh</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>緑や木を増やす</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>429</v>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Hạn chế đồ nhựa dùng một lần</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>使い捨[つかいす]て製品[せいひん]を避[さ]ける</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Hạn chế đồ nhựa dùng một lần</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>使い捨て製品を避ける</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>使い捨[つかいす]て製品[せいひん]を避[さ]ける</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Hạn chế đồ nhựa dùng một lần</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>使い捨て製品を避ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>430</v>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Chủ động chuẩn bị trước bão lũ</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>自然災害[しぜんさいがい]に普段[ふだん]から備[そな]える</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Chủ động chuẩn bị trước bão lũ</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>自然災害に普段から備える</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>自然災害[しぜんさいがい]に普段[ふだん]から備[そな]える</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Chủ động chuẩn bị trước bão lũ</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>自然災害に普段から備える</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>431</v>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Tích trữ đồ cứu hộ khẩn cấp</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>防災[ぼうさい]グッズを常備[じょうび]する</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Tích trữ đồ cứu hộ khẩn cấp</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>防災グッズを常備する</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>防災[ぼうさい]グッズを常備[じょうび]する</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>Tích trữ đồ cứu hộ khẩn cấp</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>防災グッズを常備する</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>432</v>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Ngăn chặn tình trạng ô nhiễm khí</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>大気汚染[たいきおせん]を防止[ぼうし]する</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Ngăn chặn tình trạng ô nhiễm khí</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>大気汚染を防止する</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>大気汚染[たいきおせん]を防止[ぼうし]する</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>Ngăn chặn tình trạng ô nhiễm khí</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>大気汚染を防止する</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>433</v>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Chung tay xây dựng lối sống xanh</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>持続[じぞく]可能[かのう]な暮[く]らしを実践[じっせん]する</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Chung tay xây dựng lối sống xanh</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>持続可能な暮らしを実践する</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>持続[じぞく]可能[かのう]な暮[く]らしを実践[じっせん]する</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>Chung tay xây dựng lối sống xanh</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>持続可能な暮らしを実践する</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>434</v>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Bảo vệ đa dạng sinh học</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>生物[せいぶつ]多様性[たようせい]を保全[ほぜん]する</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Bảo vệ đa dạng sinh học</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>生物多様性を保全する</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>生物[せいぶつ]多様性[たようせい]を保全[ほぜん]する</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Bảo vệ đa dạng sinh học</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>生物多様性を保全する</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>435</v>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Rời nhà sớm hơn giờ hẹn</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>早[はや]めに出発[しゅっぱつ]する</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Rời nhà sớm hơn giờ hẹn</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>早めに出発する</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>早[はや]めに出発[しゅっぱつ]する</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Rời nhà sớm hơn giờ hẹn</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>早めに出発する</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>436</v>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Luôn giữ ý thức lái xe an toàn</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>安全運転[あんぜんうんてん]を心[こころ]がける</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Luôn giữ ý thức lái xe an toàn</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>安全運転を心がける</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>安全運転[あんぜんうんてん]を心[こころ]がける</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>Luôn giữ ý thức lái xe an toàn</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>安全運転を心がける</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>437</v>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Đội mũ bảo hiểm đạt chuẩn</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>ヘルメットを正[ただ]しく着用[ちゃくよう]する</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Đội mũ bảo hiểm đạt chuẩn</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>ヘルメットを正しく着用する</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>ヘルメットを正[ただ]しく着用[ちゃくよう]する</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>Đội mũ bảo hiểm đạt chuẩn</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>ヘルメットを正しく着用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>438</v>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Tuyệt đối không vừa lái vừa dùng đt</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>ながら運転[うんてん]をしない</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Tuyệt đối không vừa lái vừa dùng đt</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>ながら運転をしない</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>ながら運転[うんてん]をしない</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>Tuyệt đối không vừa lái vừa dùng đt</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>ながら運転をしない</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>439</v>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Không vượt đèn đỏ nguy hiểm</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>信号無視[しんごうむし]をしない</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Không vượt đèn đỏ nguy hiểm</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>信号無視をしない</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>信号無視[しんごうむし]をしない</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Không vượt đèn đỏ nguy hiểm</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>信号無視をしない</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>440</v>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Ưu tiên nhường đường cho người đi bộ</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>歩行者[ほこうしゃ]を優先[ゆうせん]する</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Ưu tiên nhường đường cho người đi bộ</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>歩行者を優先する</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>歩行者[ほこうしゃ]を優先[ゆうせん]する</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Ưu tiên nhường đường cho người đi bộ</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>歩行者を優先する</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>441</v>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Tránh di chuyển vào giờ cao điểm</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ラッシュアワーを避[さ]ける</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Tránh di chuyển vào giờ cao điểm</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>ラッシュアワーを避ける</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>ラッシュアワーを避[さ]ける</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Tránh di chuyển vào giờ cao điểm</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>ラッシュアワーを避ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>442</v>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Cài dây an toàn cẩn thận trên ô tô</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>シートベルトを締[し]める</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Cài dây an toàn cẩn thận trên ô tô</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>シートベルトを締める</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>シートベルトを締[し]める</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Cài dây an toàn cẩn thận trên ô tô</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>シートベルトを締める</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>443</v>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Tận dụng vé tàu xe theo tháng</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>定期券[ていきけん]を活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Tận dụng vé tàu xe theo tháng</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>定期券を活用する</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>定期券[ていきけん]を活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Tận dụng vé tàu xe theo tháng</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>定期券を活用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>444</v>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Không tạt đầu luồn lách chen ngang</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>無理[むり]な割り込[わりこ]みをしない</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Không tạt đầu luồn lách chen ngang</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>無理な割り込みをしない</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>無理[むり]な割り込[わりこ]みをしない</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Không tạt đầu luồn lách chen ngang</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>無理な割り込みをしない</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>445</v>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Quan sát kỹ tình trạng mặt đường</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>路面状況[ろめんじょうきょう]に注意[ちゅうい]する</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Quan sát kỹ tình trạng mặt đường</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>路面状況に注意する</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>路面状況[ろめんじょうきょう]に注意[ちゅうい]する</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>Quan sát kỹ tình trạng mặt đường</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>路面状況に注意する</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>446</v>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Phát triển mạng lưới tàu điện ngầm</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>地下鉄[ちかてつ]ネットワークを整備[せいび]する</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Phát triển mạng lưới tàu điện ngầm</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>地下鉄ネットワークを整備する</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>地下鉄[ちかてつ]ネットワークを整備[せいび]する</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>Phát triển mạng lưới tàu điện ngầm</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>地下鉄ネットワークを整備する</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="n">
+        <v>447</v>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Chung tay nuôi dạy con cái</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>育児[いくじ]に協力[きょうりょく]する</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Chung tay nuôi dạy con cái</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>育児に協力する</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>育児[いくじ]に協力[きょうりょく]する</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Chung tay nuôi dạy con cái</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>育児に協力する</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>448</v>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Quản lý tài chính gia đình hợp lý</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>家計[かけい]を上手[じょうず]に管理[かんり]する</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Quản lý tài chính gia đình hợp lý</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>家計を上手に管理する</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>家計[かけい]を上手[じょうず]に管理[かんり]する</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Quản lý tài chính gia đình hợp lý</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>家計を上手に管理する</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>449</v>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Biết đặt mình vào vị trí của bạn đời</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>相手[あいて]の立場[たちば]に立[た]って考[かんが]える</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Biết đặt mình vào vị trí của bạn đời</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>相手の立場に立って考える</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>相手[あいて]の立場[たちば]に立[た]って考[かんが]える</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Biết đặt mình vào vị trí của bạn đời</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>相手の立場に立って考える</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>450</v>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Báo hiếu phụng dưỡng cha mẹ</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>親孝行[おやこうこう]をする</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Báo hiếu phụng dưỡng cha mẹ</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>親孝行をする</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>親孝行[おやこうこう]をする</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Báo hiếu phụng dưỡng cha mẹ</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>親孝行をする</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="n">
+        <v>451</v>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Tôn trọng lối sống riêng của nhau</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>互[たが]いの価値観[かちかん]を認[みと]め合[あ]う</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Tôn trọng lối sống riêng của nhau</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>互いの価値観を認め合う</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>互[たが]いの価値観[かちかん]を認[みと]め合[あ]う</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>Tôn trọng lối sống riêng của nhau</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>互いの価値観を認め合う</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="n">
+        <v>452</v>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Xây dựng tổ ấm bình yên hạnh phúc</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>温[あたた]かい家庭[かてい]を築[きづ]く</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Xây dựng tổ ấm bình yên hạnh phúc</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>温かい家庭を築く</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>温[あたた]かい家庭[かてい]を築[きづ]く</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Xây dựng tổ ấm bình yên hạnh phúc</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>温かい家庭を築く</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="n">
+        <v>453</v>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Nuôi dạy con biết yêu thương</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>思[おも]いやりの心[こころ]を育[そだ]てる</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Nuôi dạy con biết yêu thương</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>思いやりの心を育てる</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>思[おも]いやりの心[こころ]を育[そだ]てる</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Nuôi dạy con biết yêu thương</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>思いやりの心を育てる</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="n">
+        <v>454</v>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Đi bộ nhẹ nhàng mỗi ngày</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ウォーキングを習慣[しゅうかん]にする</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Đi bộ nhẹ nhàng mỗi ngày</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>ウォーキングを習慣にする</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>ウォーキングを習慣[しゅうかん]にする</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Đi bộ nhẹ nhàng mỗi ngày</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>ウォーキングを習慣にする</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>455</v>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Giãn cơ nhẹ nhàng trước khi ngủ</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>ストレッチをする</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Giãn cơ nhẹ nhàng trước khi ngủ</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>ストレッチをする</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>ストレッチをする</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Giãn cơ nhẹ nhàng trước khi ngủ</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>ストレッチをする</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>456</v>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Tăng cường sức đề kháng cho cơ thể</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>免疫力[めんえきりょく]を高[たか]める</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Tăng cường sức đề kháng cho cơ thể</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>免疫力を高める</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>免疫力[めんえきりょく]を高[たか]める</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>Tăng cường sức đề kháng cho cơ thể</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>免疫力を高める</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>457</v>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Thưởng thức đặc sản vùng miền</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>現地[げんち]の郷土料理[きょうどりょうり]を味[あじ]わう</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Thưởng thức đặc sản vùng miền</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>現地の郷土料理を味わう</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>現地[げんち]の郷土料理[きょうどりょうり]を味[あじ]わう</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>Thưởng thức đặc sản vùng miền</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>現地の郷土料理を味わう</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="n">
+        <v>458</v>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Lên lịch trình kế hoạch từ trước</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>事前[じぜん]に旅行計画[りょこうけいかく]を立[た]てる</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Lên lịch trình kế hoạch từ trước</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>事前に旅行計画を立てる</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>事前[じぜん]に旅行計画[りょこうけいかく]を立[た]てる</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>Lên lịch trình kế hoạch từ trước</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>事前に旅行計画を立てる</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>459</v>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Tham quan danh lam thắng cảnh</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>有名[ゆうめい]な観光名所[かんこうめいしょ]を巡[めぐ]る</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Tham quan danh lam thắng cảnh</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>有名な観光名所を巡る</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>有名[ゆうめい]な観光名所[かんこうめいしょ]を巡[めぐ]る</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>Tham quan danh lam thắng cảnh</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>有名な観光名所を巡る</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>460</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Gói ghém hành lý gọn gàng</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>荷物[にもつ]をコンパクトにまとめる</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Gói ghém hành lý gọn gàng</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>荷物をコンパクトにまとめる</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>荷物[にもつ]をコンパクトにまとめる</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Gói ghém hành lý gọn gàng</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>荷物をコンパクトにまとめる</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>461</v>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Lưu giữ những bức ảnh kỷ niệm đẹp</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>思い出[おもいで]の写真[しゃしん]を撮[と]る</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Lưu giữ những bức ảnh kỷ niệm đẹp</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>思い出の写真を撮る</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>思い出[おもいで]の写真[しゃしん]を撮[と]る</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>Lưu giữ những bức ảnh kỷ niệm đẹp</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>思い出の写真を撮る</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>462</v>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Trò chuyện cùng người dân địa phương</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>地元[じもと]の人[ひと]と交流[こうりゅう]する</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Trò chuyện cùng người dân địa phương</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>地元の人と交流する</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>地元[じもと]の人[ひと]と交流[こうりゅう]する</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>Trò chuyện cùng người dân địa phương</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>地元の人と交流する</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>463</v>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Chọn mua quà lưu niệm cho bạn bè</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>お土産[みやげ]を選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Chọn mua quà lưu niệm cho bạn bè</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>お土産を選ぶ</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>お土産[みやげ]を選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>Chọn mua quà lưu niệm cho bạn bè</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>お土産を選ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>464</v>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Đi chơi xa để nạp lại năng lượng</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>リフレッシュの旅[たび]に出[で]る</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Đi chơi xa để nạp lại năng lượng</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>リフレッシュの旅に出る</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>リフレッシュの旅[たび]に出[で]る</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>Đi chơi xa để nạp lại năng lượng</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>リフレッシュの旅に出る</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>465</v>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Hòa mình vào lễ hội theo mùa</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>季節[きせつ]のイベントに参加[さんか]する</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Hòa mình vào lễ hội theo mùa</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>季節のイベントに参加する</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>季節[きせつ]のイベントに参加[さんか]する</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>Hòa mình vào lễ hội theo mùa</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>季節のイベントに参加する</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>466</v>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Thăm các di tích lịch sử lâu đời</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>歴史的[れきしてき]な建造物[けんぞうぶつ]を訪[たず]ねる</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Thăm các di tích lịch sử lâu đời</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>歴史的な建造物を訪ねる</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>歴史的[れきしてき]な建造物[けんぞうぶつ]を訪[たず]ねる</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>Thăm các di tích lịch sử lâu đời</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>歴史的な建造物を訪ねる</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>467</v>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Du lịch trong phạm vi ngân sách</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>予算[よさん]内[ない]で旅[たび]を楽[たの]しむ</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Du lịch trong phạm vi ngân sách</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>予算内で旅を楽しむ</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>予算[よさん]内[ない]で旅[たび]を楽[たの]しむ</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>Du lịch trong phạm vi ngân sách</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>予算内で旅を楽しむ</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>468</v>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Rời xa nhịp sống xô bồ đô thị</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>都会[とかい]の喧騒[けんそう]を離[はな]れる</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Rời xa nhịp sống xô bồ đô thị</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>都会の喧騒を離れる</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>都会[とかい]の喧騒[けんそう]を離[はな]れる</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>Rời xa nhịp sống xô bồ đô thị</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>都会の喧騒を離れる</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>469</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Trải nghiệm cắm trại ngoài trời</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>キャンプを楽[たの]しむ</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Trải nghiệm cắm trại ngoài trời</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>キャンプを楽しむ</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>キャンプを楽[たの]しむ</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>Trải nghiệm cắm trại ngoài trời</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>キャンプを楽しむ</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>470</v>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Tích điểm thưởng thông minh</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>ポイントを賢[かしこ]く貯[た]める</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Tích điểm thưởng thông minh</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>ポイントを賢く貯める</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>ポイントを賢[かしこ]く貯[た]める</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>Tích điểm thưởng thông minh</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>ポイントを賢く貯める</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>471</v>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Tham khảo đánh giá của người mua</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>口コミ[くちこみ]やレビューを参考[さんこう]にする</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Tham khảo đánh giá của người mua</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>口コミやレビューを参考にする</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>口コミ[くちこみ]やレビューを参考[さんこう]にする</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>Tham khảo đánh giá của người mua</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>口コミやレビューを参考にする</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>472</v>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Tận dụng các đợt giảm giá lớn</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>セールや割引[わりびき]を活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Tận dụng các đợt giảm giá lớn</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>セールや割引を活用する</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>セールや割引[わりびき]を活用[かつよう]する</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>Tận dụng các đợt giảm giá lớn</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>セールや割引を活用する</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>473</v>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Ghi chép sổ chi tiêu mỗi ngày</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>家計簿[かけいぼ]をつける</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Ghi chép sổ chi tiêu mỗi ngày</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>家計簿をつける</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>家計簿[かけいぼ]をつける</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>Ghi chép sổ chi tiêu mỗi ngày</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>家計簿をつける</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>474</v>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Tận dụng đồ cũ và chợ đồ cũ</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>中古品[ちゅうこひん]やフリマアプリを使[つか]う</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Tận dụng đồ cũ và chợ đồ cũ</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>中古品やフリマアプリを使う</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>中古品[ちゅうこひん]やフリマアプリを使[つか]う</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>Tận dụng đồ cũ và chợ đồ cũ</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>中古品やフリマアプリを使う</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>475</v>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Trở thành người tiêu dùng thông thái</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>賢[かしこ]い消費者[しょうひしゃ]になる</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Trở thành người tiêu dùng thông thái</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>賢い消費者になる</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>賢[かしこ]い消費者[しょうひしゃ]になる</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>Trở thành người tiêu dùng thông thái</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>賢い消費者になる</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>476</v>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Đầu tư tiền cho trải nghiệm đáng giá</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>経験[けいけん]にお金[きん]を使[つか]う</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Đầu tư tiền cho trải nghiệm đáng giá</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>経験にお金を使う</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>経験[けいけん]にお金[きん]を使[つか]う</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>Đầu tư tiền cho trải nghiệm đáng giá</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>経験にお金を使う</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>477</v>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Tìm hiểu kỹ trước khi ký hợp đồng</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>契約内容[けいやくないよう]をしっかり読[よ]む</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Tìm hiểu kỹ trước khi ký hợp đồng</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>契約内容をしっかり読む</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>契約内容[けいやくないよう]をしっかり読[よ]む</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>Tìm hiểu kỹ trước khi ký hợp đồng</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>契約内容をしっかり読む</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>478</v>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Tránh nợ nần vượt quá khả năng</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>借金[しゃっきん]やリボ払[はら]いを避[さ]ける</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Tránh nợ nần vượt quá khả năng</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>借金やリボ払いを避ける</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>借金[しゃっきん]やリボ払[はら]いを避[さ]ける</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>Tránh nợ nần vượt quá khả năng</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>借金やリボ払いを避ける</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>479</v>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Chủ động nói chuyện bằng tiếng Nhật</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>外国語[がいこくご]で積極的[せっきょくてき]に話[はな]す</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Chủ động nói chuyện bằng tiếng Nhật</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>外国語で積極的に話す</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>外国語[がいこくご]で積極的[せっきょくてき]に話[はな]す</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>Chủ động nói chuyện bằng tiếng Nhật</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>外国語で積極的に話す</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>480</v>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Đào sâu hiểu biết văn hóa đa quốc gia</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>異文化[いぶんか]理解[りかい]を深[ふか]める</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Đào sâu hiểu biết văn hóa đa quốc gia</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>異文化理解を深める</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>異文化[いぶんか]理解[りかい]を深[ふか]める</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>Đào sâu hiểu biết văn hóa đa quốc gia</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>異文化理解を深める</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>481</v>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Luyện phương pháp đọc nhại Shadowing</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>シャドーイングを練習[れんしゅう]する</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Luyện phương pháp đọc nhại Shadowing</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>シャドーイングを練習する</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>シャドーイングを練習[れんしゅう]する</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>Luyện phương pháp đọc nhại Shadowing</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>シャドーイングを練習する</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>482</v>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Trau dồi và làm giàu vốn từ vựng</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>語彙[ごい]力[ちから]を豊[ゆた]かにする</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Trau dồi và làm giàu vốn từ vựng</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>語彙力を豊かにする</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>語彙[ごい]力[ちから]を豊[ゆた]かにする</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>Trau dồi và làm giàu vốn từ vựng</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>語彙力を豊かにする</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>483</v>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Rèn luyện kỹ năng nghe hiểu hàng ngày</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>リスニング力[ちから]を鍛[きた]える</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Rèn luyện kỹ năng nghe hiểu hàng ngày</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>リスニング力を鍛える</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>リスニング力[ちから]を鍛[きた]える</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>Rèn luyện kỹ năng nghe hiểu hàng ngày</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>リスニング力を鍛える</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>484</v>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Tham gia các khóa học online linh hoạt</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>オンライン講座[こうざ]を受講[じゅこう]する</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Tham gia các khóa học online linh hoạt</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>オンライン講座を受講する</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>オンライン講座[こうざ]を受講[じゅこう]する</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>Tham gia các khóa học online linh hoạt</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>オンライン講座を受講する</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>485</v>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Trang bị góc nhìn mang tầm quốc tế</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>グローバルな視点[してん]を持[も]つ</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Trang bị góc nhìn mang tầm quốc tế</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>グローバルな視点を持つ</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>グローバルな視点[してん]を持[も]つ</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>Trang bị góc nhìn mang tầm quốc tế</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>グローバルな視点を持つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>486</v>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Thi lấy chứng chỉ ngoại ngữ uy tín</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>検定試験[けんていしけん]に合格[ごうかく]する</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Thi lấy chứng chỉ ngoại ngữ uy tín</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>検定試験に合格する</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>検定試験[けんていしけん]に合格[ごうかく]する</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>Thi lấy chứng chỉ ngoại ngữ uy tín</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>検定試験に合格する</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>487</v>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Vượt qua rào cản ngôn ngữ để gắn kết</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>言葉[ことば]の壁[かべ]を乗り越[のりこ]える</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Vượt qua rào cản ngôn ngữ để gắn kết</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>言葉の壁を乗り越える</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>言葉[ことば]の壁[かべ]を乗り越[のりこ]える</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>Vượt qua rào cản ngôn ngữ để gắn kết</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>言葉の壁を乗り越える</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>488</v>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Tùy theo tâm trạng lúc đó để chọn</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>その時[とき]の気分[きぶん]に合[あ]わせて選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Tùy theo tâm trạng lúc đó để chọn</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>その時の気分に合わせて選ぶ</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>その時[とき]の気分[きぶん]に合[あ]わせて選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>Tùy theo tâm trạng lúc đó để chọn</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>その時の気分に合わせて選ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>489</v>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Mua của rẻ là của ôi (ham rẻ thành tốn)</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>安物買[やすものが]いの銭失[ぜにうしな]い</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Mua của rẻ là của ôi (ham rẻ thành tốn)</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>安物買いの銭失い</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>安物買[やすものが]いの銭失[ぜにうしな]い</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>Mua của rẻ là của ôi (ham rẻ thành tốn)</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>安物買いの銭失い</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>490</v>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Chọn quần áo phù hợp với bản thân</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>自分[じぶん]に合[あ]った服[ふく]を選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Chọn quần áo phù hợp với bản thân</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>自分に合った服を選ぶ</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>自分[じぶん]に合[あ]った服[ふく]を選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>Chọn quần áo phù hợp với bản thân</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>自分に合った服を選ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>491</v>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Chọn thương hiệu vì chất lượng và độ bền</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>品質[ひんしつ]と耐久性[たいきゅうせい]のためにブランドを選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Chọn thương hiệu vì chất lượng và độ bền</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>品質と耐久性のためにブランドを選ぶ</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>品質[ひんしつ]と耐久性[たいきゅうせい]のためにブランドを選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>Chọn thương hiệu vì chất lượng và độ bền</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>品質と耐久性のためにブランドを選ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>492</v>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Chọn shop uy tín và đáng tin cậy</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>信頼[しんらい]できるショップを選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Chọn shop uy tín và đáng tin cậy</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>信頼できるショップを選ぶ</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>信頼[しんらい]できるショップを選[えら]ぶ</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>Chọn shop uy tín và đáng tin cậy</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>信頼できるショップを選ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>493</v>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Hành động / có mặt trước 5 phút</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>5分前[ふんまえ]行動[こうどう]</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Hành động / có mặt trước 5 phút</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>5分前行動</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>5分前[ふんまえ]行動[こうどう]</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>Hành động / có mặt trước 5 phút</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>5分前行動</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>494</v>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Nhập gia tùy tục (tục ngữ quen thuộc)</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>郷[さと]に入[いっ]っては郷[さと]に従[したが]え</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Nhập gia tùy tục (tục ngữ quen thuộc)</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>郷に入っては郷に従え</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>郷[さと]に入[いっ]っては郷[さと]に従[したが]え</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>Nhập gia tùy tục (tục ngữ quen thuộc)</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>郷に入っては郷に従え</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16426,7 +20626,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>

</xml_diff>